<commit_message>
Soft assert for form save, faster Gmail waits, 11 AM schedule, Last_Run column, new recipients
</commit_message>
<xml_diff>
--- a/testdata/NotificationTestData.xlsx
+++ b/testdata/NotificationTestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wimate/IdeaProjects/NotificationAutomation V3/testdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wimate/IdeaProjects/NotificationAutomation V5/testdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C7381A-86A2-DA48-8EAC-9BBD8CDE30E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56D7600E-8FA7-F346-8B03-40BB70B1A321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16140" xr2:uid="{652CB739-60E5-AB45-8F25-24914DD1C0B9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="66">
   <si>
     <t>Test_ID</t>
   </si>
@@ -225,6 +225,18 @@
   </si>
   <si>
     <t>FAIL</t>
+  </si>
+  <si>
+    <t>Last_Run</t>
+  </si>
+  <si>
+    <t>14 Oct 2026, 01:48 PM</t>
+  </si>
+  <si>
+    <t>14 Oct 2026, 01:49 PM</t>
+  </si>
+  <si>
+    <t>14 Oct 2026, 01:50 PM</t>
   </si>
 </sst>
 </file>
@@ -621,7 +633,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80EDDCED-7F3B-BE4D-83F1-2B5CF55EDFE8}">
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="13.5"/>
@@ -643,9 +655,10 @@
     <col min="19" max="19" customWidth="true" width="20.0"/>
     <col min="20" max="20" customWidth="true" width="18.6640625"/>
     <col min="21" max="21" customWidth="true" width="32.5"/>
+    <col min="22" max="22" customWidth="true" width="36.33203125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -709,8 +722,11 @@
       <c r="U1" s="2" t="s">
         <v>57</v>
       </c>
+      <c r="V1" s="2" t="s">
+        <v>62</v>
+      </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" t="s" s="0">
         <v>13</v>
       </c>
@@ -774,8 +790,11 @@
       <c r="U2" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="V2" t="s" s="0">
+        <v>63</v>
+      </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" t="s" s="0">
         <v>21</v>
       </c>
@@ -839,8 +858,11 @@
       <c r="U3" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="V3" t="s" s="0">
+        <v>63</v>
+      </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" t="s" s="0">
         <v>24</v>
       </c>
@@ -904,8 +926,11 @@
       <c r="U4" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="V4" t="s" s="0">
+        <v>64</v>
+      </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" t="s" s="0">
         <v>28</v>
       </c>
@@ -969,8 +994,11 @@
       <c r="U5" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="V5" t="s" s="0">
+        <v>64</v>
+      </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" t="s" s="0">
         <v>38</v>
       </c>
@@ -1034,8 +1062,11 @@
       <c r="U6" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="V6" t="s" s="0">
+        <v>64</v>
+      </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7" t="s" s="0">
         <v>41</v>
       </c>
@@ -1099,8 +1130,11 @@
       <c r="U7" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="V7" t="s" s="0">
+        <v>65</v>
+      </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" t="s" s="0">
         <v>44</v>
       </c>
@@ -1164,8 +1198,11 @@
       <c r="U8" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="V8" t="s" s="0">
+        <v>65</v>
+      </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" t="s" s="0">
         <v>47</v>
       </c>
@@ -1229,8 +1266,11 @@
       <c r="U9" s="3" t="s">
         <v>60</v>
       </c>
+      <c r="V9" t="s" s="0">
+        <v>65</v>
+      </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="E14" t="s" s="0">
         <v>32</v>
       </c>

</xml_diff>